<commit_message>
Expand evaluation questionnaire to 15 items
Add items 11–15 and refine system responses, wording, dates and 'actos a verificar' in evaluacion/cuestionario-humano.md; update estimated time and phrasing throughout. Also update evaluacion/planilla-jueces.xlsx (judges spreadsheet). These edits extend the evaluation from 10 to 15 queries and correct/clarify several disposition references.
</commit_message>
<xml_diff>
--- a/evaluacion/planilla-jueces.xlsx
+++ b/evaluacion/planilla-jueces.xlsx
@@ -503,7 +503,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Ítems 1-10: leer la consulta y la respuesta en el cuestionario (PDF/impreso) y puntuar 1-5.</t>
+          <t>Ítems 1-15: leer la consulta y la respuesta en el cuestionario (PDF/impreso) y puntuar 1-5.</t>
         </is>
       </c>
     </row>
@@ -553,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -748,7 +748,7 @@
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>11</t>
         </is>
       </c>
       <c r="B14" s="8" t="n"/>
@@ -761,7 +761,7 @@
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B15" s="8" t="n"/>
@@ -774,7 +774,7 @@
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>13</t>
         </is>
       </c>
       <c r="B16" s="8" t="n"/>
@@ -784,60 +784,125 @@
       <c r="F16" s="8" t="n"/>
       <c r="G16" s="8" t="n"/>
     </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="n"/>
+      <c r="C17" s="8" t="n"/>
+      <c r="D17" s="8" t="n"/>
+      <c r="E17" s="8" t="n"/>
+      <c r="F17" s="8" t="n"/>
+      <c r="G17" s="8" t="n"/>
+    </row>
     <row r="18">
-      <c r="A18" s="9" t="inlineStr">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="B18" s="8" t="n"/>
+      <c r="C18" s="8" t="n"/>
+      <c r="D18" s="8" t="n"/>
+      <c r="E18" s="8" t="n"/>
+      <c r="F18" s="8" t="n"/>
+      <c r="G18" s="8" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B19" s="8" t="n"/>
+      <c r="C19" s="8" t="n"/>
+      <c r="D19" s="8" t="n"/>
+      <c r="E19" s="8" t="n"/>
+      <c r="F19" s="8" t="n"/>
+      <c r="G19" s="8" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="B20" s="8" t="n"/>
+      <c r="C20" s="8" t="n"/>
+      <c r="D20" s="8" t="n"/>
+      <c r="E20" s="8" t="n"/>
+      <c r="F20" s="8" t="n"/>
+      <c r="G20" s="8" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B21" s="8" t="n"/>
+      <c r="C21" s="8" t="n"/>
+      <c r="D21" s="8" t="n"/>
+      <c r="E21" s="8" t="n"/>
+      <c r="F21" s="8" t="n"/>
+      <c r="G21" s="8" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="9" t="inlineStr">
         <is>
           <t>Bloque final (1-5)</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="10" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="10" t="inlineStr">
         <is>
           <t>Confianza</t>
         </is>
       </c>
-      <c r="B19" s="8" t="n"/>
-      <c r="C19" s="5" t="inlineStr">
+      <c r="B24" s="8" t="n"/>
+      <c r="C24" s="5" t="inlineStr">
         <is>
           <t>Me apoyaría en este sistema para consultas de mi trabajo/estudio</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="10" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="10" t="inlineStr">
         <is>
           <t>Ventaja</t>
         </is>
       </c>
-      <c r="B20" s="8" t="n"/>
-      <c r="C20" s="5" t="inlineStr">
+      <c r="B25" s="8" t="n"/>
+      <c r="C25" s="5" t="inlineStr">
         <is>
           <t>Me resulta mejor que la forma en que hoy busco normativa</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="10" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="10" t="inlineStr">
         <is>
           <t>Adopción</t>
         </is>
       </c>
-      <c r="B21" s="8" t="n"/>
-      <c r="C21" s="5" t="inlineStr">
+      <c r="B26" s="8" t="n"/>
+      <c r="C26" s="5" t="inlineStr">
         <is>
           <t>Recomendaría que la Universidad lo ofrezca abiertamente</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="10" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="10" t="inlineStr">
         <is>
           <t>Comentario libre</t>
         </is>
       </c>
-      <c r="B22" s="8" t="n"/>
-      <c r="C22" s="5" t="inlineStr">
+      <c r="B27" s="8" t="n"/>
+      <c r="C27" s="5" t="inlineStr">
         <is>
           <t>Qué te sorprendió, qué le falta, qué no le creíste</t>
         </is>
@@ -845,11 +910,11 @@
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation sqref="B4:E16 B19:B21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Puntaje" error="Entre 1 y 5" type="whole" operator="between">
+    <dataValidation sqref="B4:E21 B24:B26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Puntaje" error="Entre 1 y 5" type="whole" operator="between">
       <formula1>1</formula1>
       <formula2>5</formula2>
     </dataValidation>
-    <dataValidation sqref="F4:F16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F4:F21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"SÍ,NO"</formula1>
     </dataValidation>
   </dataValidations>
@@ -863,7 +928,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1058,7 +1123,7 @@
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>11</t>
         </is>
       </c>
       <c r="B14" s="8" t="n"/>
@@ -1071,7 +1136,7 @@
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B15" s="8" t="n"/>
@@ -1084,7 +1149,7 @@
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>13</t>
         </is>
       </c>
       <c r="B16" s="8" t="n"/>
@@ -1094,60 +1159,125 @@
       <c r="F16" s="8" t="n"/>
       <c r="G16" s="8" t="n"/>
     </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="n"/>
+      <c r="C17" s="8" t="n"/>
+      <c r="D17" s="8" t="n"/>
+      <c r="E17" s="8" t="n"/>
+      <c r="F17" s="8" t="n"/>
+      <c r="G17" s="8" t="n"/>
+    </row>
     <row r="18">
-      <c r="A18" s="9" t="inlineStr">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="B18" s="8" t="n"/>
+      <c r="C18" s="8" t="n"/>
+      <c r="D18" s="8" t="n"/>
+      <c r="E18" s="8" t="n"/>
+      <c r="F18" s="8" t="n"/>
+      <c r="G18" s="8" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B19" s="8" t="n"/>
+      <c r="C19" s="8" t="n"/>
+      <c r="D19" s="8" t="n"/>
+      <c r="E19" s="8" t="n"/>
+      <c r="F19" s="8" t="n"/>
+      <c r="G19" s="8" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="B20" s="8" t="n"/>
+      <c r="C20" s="8" t="n"/>
+      <c r="D20" s="8" t="n"/>
+      <c r="E20" s="8" t="n"/>
+      <c r="F20" s="8" t="n"/>
+      <c r="G20" s="8" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B21" s="8" t="n"/>
+      <c r="C21" s="8" t="n"/>
+      <c r="D21" s="8" t="n"/>
+      <c r="E21" s="8" t="n"/>
+      <c r="F21" s="8" t="n"/>
+      <c r="G21" s="8" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="9" t="inlineStr">
         <is>
           <t>Bloque final (1-5)</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="10" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="10" t="inlineStr">
         <is>
           <t>Confianza</t>
         </is>
       </c>
-      <c r="B19" s="8" t="n"/>
-      <c r="C19" s="5" t="inlineStr">
+      <c r="B24" s="8" t="n"/>
+      <c r="C24" s="5" t="inlineStr">
         <is>
           <t>Me apoyaría en este sistema para consultas de mi trabajo/estudio</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="10" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="10" t="inlineStr">
         <is>
           <t>Ventaja</t>
         </is>
       </c>
-      <c r="B20" s="8" t="n"/>
-      <c r="C20" s="5" t="inlineStr">
+      <c r="B25" s="8" t="n"/>
+      <c r="C25" s="5" t="inlineStr">
         <is>
           <t>Me resulta mejor que la forma en que hoy busco normativa</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="10" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="10" t="inlineStr">
         <is>
           <t>Adopción</t>
         </is>
       </c>
-      <c r="B21" s="8" t="n"/>
-      <c r="C21" s="5" t="inlineStr">
+      <c r="B26" s="8" t="n"/>
+      <c r="C26" s="5" t="inlineStr">
         <is>
           <t>Recomendaría que la Universidad lo ofrezca abiertamente</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="10" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="10" t="inlineStr">
         <is>
           <t>Comentario libre</t>
         </is>
       </c>
-      <c r="B22" s="8" t="n"/>
-      <c r="C22" s="5" t="inlineStr">
+      <c r="B27" s="8" t="n"/>
+      <c r="C27" s="5" t="inlineStr">
         <is>
           <t>Qué te sorprendió, qué le falta, qué no le creíste</t>
         </is>
@@ -1155,11 +1285,11 @@
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation sqref="B4:E16 B19:B21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Puntaje" error="Entre 1 y 5" type="whole" operator="between">
+    <dataValidation sqref="B4:E21 B24:B26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Puntaje" error="Entre 1 y 5" type="whole" operator="between">
       <formula1>1</formula1>
       <formula2>5</formula2>
     </dataValidation>
-    <dataValidation sqref="F4:F16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F4:F21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"SÍ,NO"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1173,7 +1303,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1368,7 +1498,7 @@
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>11</t>
         </is>
       </c>
       <c r="B14" s="8" t="n"/>
@@ -1381,7 +1511,7 @@
     <row r="15">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>P2</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B15" s="8" t="n"/>
@@ -1394,7 +1524,7 @@
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>P3</t>
+          <t>13</t>
         </is>
       </c>
       <c r="B16" s="8" t="n"/>
@@ -1404,60 +1534,125 @@
       <c r="F16" s="8" t="n"/>
       <c r="G16" s="8" t="n"/>
     </row>
+    <row r="17">
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="n"/>
+      <c r="C17" s="8" t="n"/>
+      <c r="D17" s="8" t="n"/>
+      <c r="E17" s="8" t="n"/>
+      <c r="F17" s="8" t="n"/>
+      <c r="G17" s="8" t="n"/>
+    </row>
     <row r="18">
-      <c r="A18" s="9" t="inlineStr">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="B18" s="8" t="n"/>
+      <c r="C18" s="8" t="n"/>
+      <c r="D18" s="8" t="n"/>
+      <c r="E18" s="8" t="n"/>
+      <c r="F18" s="8" t="n"/>
+      <c r="G18" s="8" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="B19" s="8" t="n"/>
+      <c r="C19" s="8" t="n"/>
+      <c r="D19" s="8" t="n"/>
+      <c r="E19" s="8" t="n"/>
+      <c r="F19" s="8" t="n"/>
+      <c r="G19" s="8" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="B20" s="8" t="n"/>
+      <c r="C20" s="8" t="n"/>
+      <c r="D20" s="8" t="n"/>
+      <c r="E20" s="8" t="n"/>
+      <c r="F20" s="8" t="n"/>
+      <c r="G20" s="8" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="7" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="B21" s="8" t="n"/>
+      <c r="C21" s="8" t="n"/>
+      <c r="D21" s="8" t="n"/>
+      <c r="E21" s="8" t="n"/>
+      <c r="F21" s="8" t="n"/>
+      <c r="G21" s="8" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="9" t="inlineStr">
         <is>
           <t>Bloque final (1-5)</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="10" t="inlineStr">
+    <row r="24">
+      <c r="A24" s="10" t="inlineStr">
         <is>
           <t>Confianza</t>
         </is>
       </c>
-      <c r="B19" s="8" t="n"/>
-      <c r="C19" s="5" t="inlineStr">
+      <c r="B24" s="8" t="n"/>
+      <c r="C24" s="5" t="inlineStr">
         <is>
           <t>Me apoyaría en este sistema para consultas de mi trabajo/estudio</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="10" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="10" t="inlineStr">
         <is>
           <t>Ventaja</t>
         </is>
       </c>
-      <c r="B20" s="8" t="n"/>
-      <c r="C20" s="5" t="inlineStr">
+      <c r="B25" s="8" t="n"/>
+      <c r="C25" s="5" t="inlineStr">
         <is>
           <t>Me resulta mejor que la forma en que hoy busco normativa</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="10" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="10" t="inlineStr">
         <is>
           <t>Adopción</t>
         </is>
       </c>
-      <c r="B21" s="8" t="n"/>
-      <c r="C21" s="5" t="inlineStr">
+      <c r="B26" s="8" t="n"/>
+      <c r="C26" s="5" t="inlineStr">
         <is>
           <t>Recomendaría que la Universidad lo ofrezca abiertamente</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="10" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="10" t="inlineStr">
         <is>
           <t>Comentario libre</t>
         </is>
       </c>
-      <c r="B22" s="8" t="n"/>
-      <c r="C22" s="5" t="inlineStr">
+      <c r="B27" s="8" t="n"/>
+      <c r="C27" s="5" t="inlineStr">
         <is>
           <t>Qué te sorprendió, qué le falta, qué no le creíste</t>
         </is>
@@ -1465,11 +1660,11 @@
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation sqref="B4:E16 B19:B21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Puntaje" error="Entre 1 y 5" type="whole" operator="between">
+    <dataValidation sqref="B4:E21 B24:B26" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" errorTitle="Puntaje" error="Entre 1 y 5" type="whole" operator="between">
       <formula1>1</formula1>
       <formula2>5</formula2>
     </dataValidation>
-    <dataValidation sqref="F4:F16" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="F4:F21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"SÍ,NO"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Add licdia deployment, eval data, and frontend tweaks
Add deployment supporting files for licdia (systemd service, nginx snippet, and README). Add a built frontend under frontend/dist-licdia and adjust frontend sources to compute API base (API_BASE) and use BASE relative paths; set Vite base to './' and make default logo path respect BASE_URL. Reorganize evaluation: move automated evaluation scripts/data to evaluacion_automatica/, add human-eval artifacts and a compiler script (evaluacion/compilar_respuestas.py), and update questionnaire and judge responses. Update paper sources and regenerated LaTeX build artifacts (bibliography and minor text/figure changes). Misc: small README clarifications.
</commit_message>
<xml_diff>
--- a/evaluacion/planilla-jueces.xlsx
+++ b/evaluacion/planilla-jueces.xlsx
@@ -553,7 +553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -850,59 +850,13 @@
       <c r="G21" s="8" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="9" t="inlineStr">
-        <is>
-          <t>Bloque final (1-5)</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="10" t="inlineStr">
-        <is>
-          <t>Confianza</t>
-        </is>
-      </c>
-      <c r="B24" s="8" t="n"/>
-      <c r="C24" s="5" t="inlineStr">
-        <is>
-          <t>Me apoyaría en este sistema para consultas de mi trabajo/estudio</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="10" t="inlineStr">
-        <is>
-          <t>Ventaja</t>
-        </is>
-      </c>
-      <c r="B25" s="8" t="n"/>
-      <c r="C25" s="5" t="inlineStr">
-        <is>
-          <t>Me resulta mejor que la forma en que hoy busco normativa</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="10" t="inlineStr">
-        <is>
-          <t>Adopción</t>
-        </is>
-      </c>
-      <c r="B26" s="8" t="n"/>
-      <c r="C26" s="5" t="inlineStr">
-        <is>
-          <t>Recomendaría que la Universidad lo ofrezca abiertamente</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="10" t="inlineStr">
+      <c r="A23" s="10" t="inlineStr">
         <is>
           <t>Comentario libre</t>
         </is>
       </c>
-      <c r="B27" s="8" t="n"/>
-      <c r="C27" s="5" t="inlineStr">
+      <c r="B23" s="8" t="n"/>
+      <c r="C23" s="5" t="inlineStr">
         <is>
           <t>Qué te sorprendió, qué le falta, qué no le creíste</t>
         </is>
@@ -928,7 +882,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1225,59 +1179,13 @@
       <c r="G21" s="8" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="9" t="inlineStr">
-        <is>
-          <t>Bloque final (1-5)</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="10" t="inlineStr">
-        <is>
-          <t>Confianza</t>
-        </is>
-      </c>
-      <c r="B24" s="8" t="n"/>
-      <c r="C24" s="5" t="inlineStr">
-        <is>
-          <t>Me apoyaría en este sistema para consultas de mi trabajo/estudio</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="10" t="inlineStr">
-        <is>
-          <t>Ventaja</t>
-        </is>
-      </c>
-      <c r="B25" s="8" t="n"/>
-      <c r="C25" s="5" t="inlineStr">
-        <is>
-          <t>Me resulta mejor que la forma en que hoy busco normativa</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="10" t="inlineStr">
-        <is>
-          <t>Adopción</t>
-        </is>
-      </c>
-      <c r="B26" s="8" t="n"/>
-      <c r="C26" s="5" t="inlineStr">
-        <is>
-          <t>Recomendaría que la Universidad lo ofrezca abiertamente</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="10" t="inlineStr">
+      <c r="A23" s="10" t="inlineStr">
         <is>
           <t>Comentario libre</t>
         </is>
       </c>
-      <c r="B27" s="8" t="n"/>
-      <c r="C27" s="5" t="inlineStr">
+      <c r="B23" s="8" t="n"/>
+      <c r="C23" s="5" t="inlineStr">
         <is>
           <t>Qué te sorprendió, qué le falta, qué no le creíste</t>
         </is>
@@ -1303,7 +1211,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -1600,59 +1508,13 @@
       <c r="G21" s="8" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="9" t="inlineStr">
-        <is>
-          <t>Bloque final (1-5)</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="10" t="inlineStr">
-        <is>
-          <t>Confianza</t>
-        </is>
-      </c>
-      <c r="B24" s="8" t="n"/>
-      <c r="C24" s="5" t="inlineStr">
-        <is>
-          <t>Me apoyaría en este sistema para consultas de mi trabajo/estudio</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="10" t="inlineStr">
-        <is>
-          <t>Ventaja</t>
-        </is>
-      </c>
-      <c r="B25" s="8" t="n"/>
-      <c r="C25" s="5" t="inlineStr">
-        <is>
-          <t>Me resulta mejor que la forma en que hoy busco normativa</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="10" t="inlineStr">
-        <is>
-          <t>Adopción</t>
-        </is>
-      </c>
-      <c r="B26" s="8" t="n"/>
-      <c r="C26" s="5" t="inlineStr">
-        <is>
-          <t>Recomendaría que la Universidad lo ofrezca abiertamente</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="10" t="inlineStr">
+      <c r="A23" s="10" t="inlineStr">
         <is>
           <t>Comentario libre</t>
         </is>
       </c>
-      <c r="B27" s="8" t="n"/>
-      <c r="C27" s="5" t="inlineStr">
+      <c r="B23" s="8" t="n"/>
+      <c r="C23" s="5" t="inlineStr">
         <is>
           <t>Qué te sorprendió, qué le falta, qué no le creíste</t>
         </is>

</xml_diff>